<commit_message>
Actualizacion automatica del mapa (2026-06-01 13:21:02)
</commit_message>
<xml_diff>
--- a/mapa_interactivo_Optical_Power.xlsx
+++ b/mapa_interactivo_Optical_Power.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N9"/>
+  <dimension ref="A1:N26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -611,25 +611,25 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>S00392154</t>
+          <t>S00472155</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>4/20/2026</t>
+          <t>4/29/2026</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>MOLDES 3802</t>
+          <t>MARTI, JOSE 3124</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t xml:space="preserve">03863625 </t>
+          <t xml:space="preserve">04033967 </t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -644,7 +644,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>NORMALIZAR CABLES FUERA DE NORMA</t>
+          <t>NORMALIZAR CABLES A BAJA ALTURA</t>
         </is>
       </c>
       <c r="I4" t="n">
@@ -652,48 +652,48 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>{"direccionesNormalizadas": [{"altura": 3802, "cod_calle": 13099, "cod_calle_cruce": null, "cod_partido": "caba", "coordenadas": {"srid": 4326, "x": "-58.472225", "y": "-34.548862"}, "direccion": "MOLDES 3802, CABA", "nombre_calle": "MOLDES", "nombre_calle_cruce": "", "nombre_localidad": "CABA", "nombre_partido": "CABA", "tipo": "calle_altura"}]}</t>
+          <t>{"direccionesNormalizadas": [{"altura": 3124, "cod_calle": 13034, "cod_calle_cruce": null, "cod_partido": "caba", "coordenadas": {"srid": 4326, "x": "-58.442102", "y": "-34.661270"}, "direccion": "MARTI, JOSE 3124, CABA", "nombre_calle": "MARTI, JOSE", "nombre_calle_cruce": "", "nombre_localidad": "CABA", "nombre_partido": "CABA", "tipo": "calle_altura"}]}</t>
         </is>
       </c>
       <c r="K4" t="n">
-        <v>-58.472225</v>
+        <v>-58.442102</v>
       </c>
       <c r="L4" t="n">
-        <v>-34.548862</v>
+        <v>-34.66127</v>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>Saavedra</t>
+          <t>San Telmo</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>S00410561</t>
+          <t>9073</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>4/20/2026</t>
+          <t>4/30/2026</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>ANDONAEGUI 1824</t>
+          <t>EL SALVADOR 5897</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t xml:space="preserve">03863944 </t>
+          <t>PENDIENTE ADMIN</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -708,7 +708,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>NORMALIZAR CABLES SOBRE LA FACHADA</t>
+          <t>NORMALIZAR CABLES A BAJA ALTURA</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -716,48 +716,48 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>{"direccionesNormalizadas": [{"altura": 1824, "cod_calle": 1082, "cod_calle_cruce": null, "cod_partido": "caba", "coordenadas": {"srid": 4326, "x": "-58.484495", "y": "-34.581735"}, "direccion": "ANDONAEGUI 1824, CABA", "nombre_calle": "ANDONAEGUI", "nombre_calle_cruce": "", "nombre_localidad": "CABA", "nombre_partido": "CABA", "tipo": "calle_altura"}]}</t>
+          <t>{"direccionesNormalizadas": [{"altura": 5897, "cod_calle": 5050, "cod_calle_cruce": null, "cod_partido": "caba", "coordenadas": {"srid": 4326, "x": "-58.438216", "y": "-34.580964"}, "direccion": "EL SALVADOR 5897, CABA", "nombre_calle": "EL SALVADOR", "nombre_calle_cruce": "", "nombre_localidad": "CABA", "nombre_partido": "CABA", "tipo": "calle_altura"}]}</t>
         </is>
       </c>
       <c r="K5" t="n">
-        <v>-58.484495</v>
+        <v>-58.438216</v>
       </c>
       <c r="L5" t="n">
-        <v>-34.581735</v>
+        <v>-34.580964</v>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>Palermo</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>S00415175</t>
+          <t>9094</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>4/20/2026</t>
+          <t>5/10/2026</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>ARANGUREN, JUAN F., DR. 4894</t>
+          <t>CARRIL, SALVADOR MARIA DEL AV. 3236</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t xml:space="preserve">03864108 </t>
+          <t>PENDIENTE ADMIN</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -780,18 +780,18 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>{"direccionesNormalizadas": [{"altura": 4894, "cod_calle": 1094, "cod_calle_cruce": null, "cod_partido": "caba", "coordenadas": {"srid": 4326, "x": "-58.495815", "y": "-34.632491"}, "direccion": "ARANGUREN, JUAN F., DR. 4894, CABA", "nombre_calle": "ARANGUREN, JUAN F., DR.", "nombre_calle_cruce": "", "nombre_localidad": "CABA", "nombre_partido": "CABA", "tipo": "calle_altura"}]}</t>
+          <t>{"direccionesNormalizadas": [{"altura": 3236, "cod_calle": 4039, "cod_calle_cruce": null, "cod_partido": "caba", "coordenadas": {"srid": 4326, "x": "-58.502582", "y": "-34.593476"}, "direccion": "CARRIL, SALVADOR MARIA DEL AV. 3236, CABA", "nombre_calle": "CARRIL, SALVADOR MARIA DEL AV.", "nombre_calle_cruce": "", "nombre_localidad": "CABA", "nombre_partido": "CABA", "tipo": "calle_altura"}]}</t>
         </is>
       </c>
       <c r="K6" t="n">
-        <v>-58.495815</v>
+        <v>-58.502582</v>
       </c>
       <c r="L6" t="n">
-        <v>-34.632491</v>
+        <v>-34.593476</v>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Paternal</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
@@ -803,17 +803,17 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>9032</t>
+          <t>9128</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>4/24/2026</t>
+          <t>5/10/2026</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>CERETTI 2089</t>
+          <t>ECHEVERRIA 5596</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -821,7 +821,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>SE GENERA OT POR PEX</t>
+          <t>PENDIENTE ADMIN</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -836,7 +836,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>NORMALIZAR CABLES BAJOS</t>
+          <t>NORMALIZAR CABLES A BAJA ALTURA</t>
         </is>
       </c>
       <c r="I7" t="n">
@@ -844,14 +844,14 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>{"direccionesNormalizadas": [{"altura": 2089, "cod_calle": 3115, "cod_calle_cruce": null, "cod_partido": "caba", "coordenadas": {"srid": 4326, "x": "-58.490439", "y": "-34.581351"}, "direccion": "CERETTI 2089, CABA", "nombre_calle": "CERETTI", "nombre_calle_cruce": "", "nombre_localidad": "CABA", "nombre_partido": "CABA", "tipo": "calle_altura"}]}</t>
+          <t>{"direccionesNormalizadas": [{"altura": 5596, "cod_calle": 5007, "cod_calle_cruce": null, "cod_partido": "caba", "coordenadas": {"srid": 4326, "x": "-58.486598", "y": "-34.582134"}, "direccion": "ECHEVERRIA 5596, CABA", "nombre_calle": "ECHEVERRIA", "nombre_calle_cruce": "", "nombre_localidad": "CABA", "nombre_partido": "CABA", "tipo": "calle_altura"}]}</t>
         </is>
       </c>
       <c r="K7" t="n">
-        <v>-58.490439</v>
+        <v>-58.486598</v>
       </c>
       <c r="L7" t="n">
-        <v>-34.581351</v>
+        <v>-34.582134</v>
       </c>
       <c r="M7" t="inlineStr">
         <is>
@@ -867,25 +867,25 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>S00421935</t>
+          <t xml:space="preserve">9141 </t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>4/24/2026</t>
+          <t>5/13/2026</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>INDEPENDENCIA AV. 741</t>
+          <t>CUBAS, JOSE 4440</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>3</v>
+        <v>13</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>SE GENERA OT POR PEX</t>
+          <t>PENDIENTE ADMIN</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -900,7 +900,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>NORMALIZAR CABLES A BAJA ALTURA</t>
+          <t>DESMONTAR CABLES CORTADOS Y DESMONTAR POSTE INCLINADO</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -908,48 +908,48 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>{"direccionesNormalizadas": [{"altura": 741, "cod_calle": 9010, "cod_calle_cruce": null, "cod_partido": "caba", "coordenadas": {"srid": 4326, "x": "-58.376567", "y": "-34.617309"}, "direccion": "INDEPENDENCIA AV. 741, CABA", "nombre_calle": "INDEPENDENCIA AV.", "nombre_calle_cruce": "", "nombre_localidad": "CABA", "nombre_partido": "CABA", "tipo": "calle_altura"}]}</t>
+          <t>{"direccionesNormalizadas": [{"altura": 4440, "cod_calle": 3198, "cod_calle_cruce": null, "cod_partido": "caba", "coordenadas": {"srid": 4326, "x": "-58.519391", "y": "-34.600472"}, "direccion": "CUBAS, JOSE 4440, CABA", "nombre_calle": "CUBAS, JOSE", "nombre_calle_cruce": "", "nombre_localidad": "CABA", "nombre_partido": "CABA", "tipo": "calle_altura"}]}</t>
         </is>
       </c>
       <c r="K8" t="n">
-        <v>-58.376567</v>
+        <v>-58.519391</v>
       </c>
       <c r="L8" t="n">
-        <v>-34.617309</v>
+        <v>-34.600472</v>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>San Telmo</t>
+          <t>Paternal</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>S00472155</t>
+          <t>S00347551</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>4/29/2026</t>
+          <t>5/13/2026</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>MARTI, JOSE 3124</t>
+          <t>BILBAO, FRANCISCO 2124</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>SE GENERA OT POR PEX</t>
+          <t>PENDIENTE ADMIN</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -972,21 +972,1109 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>{"direccionesNormalizadas": [{"altura": 3124, "cod_calle": 13034, "cod_calle_cruce": null, "cod_partido": "caba", "coordenadas": {"srid": 4326, "x": "-58.442102", "y": "-34.661270"}, "direccion": "MARTI, JOSE 3124, CABA", "nombre_calle": "MARTI, JOSE", "nombre_calle_cruce": "", "nombre_localidad": "CABA", "nombre_partido": "CABA", "tipo": "calle_altura"}]}</t>
+          <t>{"direccionesNormalizadas": [{"altura": 2124, "cod_calle": 2081, "cod_calle_cruce": null, "cod_partido": "caba", "coordenadas": {"srid": 4326, "x": "-58.456407", "y": "-34.633376"}, "direccion": "BILBAO, FRANCISCO 2124, CABA", "nombre_calle": "BILBAO, FRANCISCO", "nombre_calle_cruce": "", "nombre_localidad": "CABA", "nombre_partido": "CABA", "tipo": "calle_altura"}]}</t>
         </is>
       </c>
       <c r="K9" t="n">
-        <v>-58.442102</v>
+        <v>-58.456407</v>
       </c>
       <c r="L9" t="n">
-        <v>-34.66127</v>
+        <v>-34.633376</v>
       </c>
       <c r="M9" t="inlineStr">
         <is>
+          <t>Boedo</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>S00415298</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>5/13/2026</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>CARDOSO 17</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>10</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>PENDIENTE ADMIN</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Optical Power</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>NORMALIZAR TENDIDO A BAJA ALTURA</t>
+        </is>
+      </c>
+      <c r="I10" t="n">
+        <v>1</v>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>{"direccionesNormalizadas": [{"altura": 17, "cod_calle": 3070, "cod_calle_cruce": null, "cod_partido": "caba", "coordenadas": {"srid": 4326, "x": "-58.492138", "y": "-34.635993"}, "direccion": "CARDOSO 17, CABA", "nombre_calle": "CARDOSO", "nombre_calle_cruce": "", "nombre_localidad": "CABA", "nombre_partido": "CABA", "tipo": "calle_altura"}]}</t>
+        </is>
+      </c>
+      <c r="K10" t="n">
+        <v>-58.492138</v>
+      </c>
+      <c r="L10" t="n">
+        <v>-34.635993</v>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>Devoto</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>Capital Norte</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>S00435575</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>5/13/2026</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>LAMAS, ANDRES 1720</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>11</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>PENDIENTE ADMIN</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Optical Power</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>NORMALIZAR CABLES A BAJA ALTURA</t>
+        </is>
+      </c>
+      <c r="I11" t="n">
+        <v>1</v>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>{"direccionesNormalizadas": [{"altura": 1720, "cod_calle": 12040, "cod_calle_cruce": null, "cod_partido": "caba", "coordenadas": {"srid": 4326, "x": "-58.467729", "y": "-34.609182"}, "direccion": "LAMAS, ANDRES 1720, CABA", "nombre_calle": "LAMAS, ANDRES", "nombre_calle_cruce": "", "nombre_localidad": "CABA", "nombre_partido": "CABA", "tipo": "calle_altura"}]}</t>
+        </is>
+      </c>
+      <c r="K11" t="n">
+        <v>-58.467729</v>
+      </c>
+      <c r="L11" t="n">
+        <v>-34.609182</v>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>Paternal</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>Capital Norte</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>S00456441</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>5/13/2026</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>QUESADA 4154</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>12</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>PENDIENTE ADMIN</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Optical Power</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>CORTAR CABLES EN DESUSO Y VERIFICAR ESTADO COLUMNA, DOCUMENTAR CON FOTOS</t>
+        </is>
+      </c>
+      <c r="I12" t="n">
+        <v>1</v>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>{"direccionesNormalizadas": [{"altura": 4154, "cod_calle": 18005, "cod_calle_cruce": null, "cod_partido": "caba", "coordenadas": {"srid": 4326, "x": "-58.481018", "y": "-34.563694"}, "direccion": "QUESADA 4154, CABA", "nombre_calle": "QUESADA", "nombre_calle_cruce": "", "nombre_localidad": "CABA", "nombre_partido": "CABA", "tipo": "calle_altura"}]}</t>
+        </is>
+      </c>
+      <c r="K12" t="n">
+        <v>-58.481018</v>
+      </c>
+      <c r="L12" t="n">
+        <v>-34.563694</v>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>Saavedra</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>Capital Norte</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">9153 </t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>5/14/2026</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>ALVAREZ THOMAS AV. 1720</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>15</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>PENDIENTE ADMIN</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Optical Power</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>NORMALIZAR CABLES A BAJA ALTURA</t>
+        </is>
+      </c>
+      <c r="I13" t="n">
+        <v>1</v>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>{"direccionesNormalizadas": [{"altura": 1720, "cod_calle": 1059, "cod_calle_cruce": null, "cod_partido": "caba", "coordenadas": {"srid": 4326, "x": "-58.466347", "y": "-34.579162"}, "direccion": "ALVAREZ THOMAS AV. 1720, CABA", "nombre_calle": "ALVAREZ THOMAS AV.", "nombre_calle_cruce": "", "nombre_localidad": "CABA", "nombre_partido": "CABA", "tipo": "calle_altura"}]}</t>
+        </is>
+      </c>
+      <c r="K13" t="n">
+        <v>-58.466347</v>
+      </c>
+      <c r="L13" t="n">
+        <v>-34.579162</v>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>Colegiales</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>Capital Norte</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">9158 </t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>5/13/2026</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>FRANCO 2415</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>15</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>PENDIENTE ADMIN</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Optical Power</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>MORMALIZAR TENDIDO A BAJA ALTURA</t>
+        </is>
+      </c>
+      <c r="I14" t="n">
+        <v>1</v>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>{"direccionesNormalizadas": [{"altura": 2415, "cod_calle": 6052, "cod_calle_cruce": null, "cod_partido": "caba", "coordenadas": {"srid": 4326, "x": "-58.501083", "y": "-34.578059"}, "direccion": "FRANCO 2415, CABA", "nombre_calle": "FRANCO", "nombre_calle_cruce": "", "nombre_localidad": "CABA", "nombre_partido": "CABA", "tipo": "calle_altura"}]}</t>
+        </is>
+      </c>
+      <c r="K14" t="n">
+        <v>-58.501083</v>
+      </c>
+      <c r="L14" t="n">
+        <v>-34.578059</v>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>Paternal</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>Capital Norte</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">9159 </t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>5/13/2026</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>BAZURCO 2442</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>12</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>PENDIENTE ADMIN</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Optical Power</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>NORMALIZAR TENDIDO A BAJA ALTURA</t>
+        </is>
+      </c>
+      <c r="I15" t="n">
+        <v>1</v>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>{"direccionesNormalizadas": [{"altura": 2442, "cod_calle": 2038, "cod_calle_cruce": null, "cod_partido": "caba", "coordenadas": {"srid": 4326, "x": "-58.502043", "y": "-34.577603"}, "direccion": "BAZURCO 2442, CABA", "nombre_calle": "BAZURCO", "nombre_calle_cruce": "", "nombre_localidad": "CABA", "nombre_partido": "CABA", "tipo": "calle_altura"}]}</t>
+        </is>
+      </c>
+      <c r="K15" t="n">
+        <v>-58.502043</v>
+      </c>
+      <c r="L15" t="n">
+        <v>-34.577603</v>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>Paternal</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>Capital Norte</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>9160</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>5/13/2026</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>CARACAS 5377</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>12</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>PENDIENTE ADMIN</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Optical Power</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>NORMALIZAR RED A BAJA ALTURA</t>
+        </is>
+      </c>
+      <c r="I16" t="n">
+        <v>1</v>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>{"direccionesNormalizadas": [{"altura": 5377, "cod_calle": 3062, "cod_calle_cruce": null, "cod_partido": "caba", "coordenadas": {"srid": 4326, "x": "-58.500199", "y": "-34.576706"}, "direccion": "CARACAS 5377, CABA", "nombre_calle": "CARACAS", "nombre_calle_cruce": "", "nombre_localidad": "CABA", "nombre_partido": "CABA", "tipo": "calle_altura"}]}</t>
+        </is>
+      </c>
+      <c r="K16" t="n">
+        <v>-58.500199</v>
+      </c>
+      <c r="L16" t="n">
+        <v>-34.576706</v>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>Paternal</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>Capital Norte</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">9185 </t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>5/13/2026</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>CAMARGO 1157</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>15</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>PENDIENTE ADMIN</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Optical Power</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>NORMALIZAR RED A BAJA ALTURA</t>
+        </is>
+      </c>
+      <c r="I17" t="n">
+        <v>1</v>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>{"direccionesNormalizadas": [{"altura": 1157, "cod_calle": 3033, "cod_calle_cruce": null, "cod_partido": "caba", "coordenadas": {"srid": 4326, "x": "-58.445853", "y": "-34.595224"}, "direccion": "CAMARGO 1157, CABA", "nombre_calle": "CAMARGO", "nombre_calle_cruce": "", "nombre_localidad": "CABA", "nombre_partido": "CABA", "tipo": "calle_altura"}]}</t>
+        </is>
+      </c>
+      <c r="K17" t="n">
+        <v>-58.445853</v>
+      </c>
+      <c r="L17" t="n">
+        <v>-34.595224</v>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>Paternal</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>Capital Norte</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">9188 </t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>5/13/2026</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>BARZANA 1566</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>12</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>PENDIENTE ADMIN</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Optical Power</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>NORMALIZAR RED A BAJA ALTURA</t>
+        </is>
+      </c>
+      <c r="I18" t="n">
+        <v>1</v>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>{"direccionesNormalizadas": [{"altura": 1566, "cod_calle": 2023, "cod_calle_cruce": null, "cod_partido": "caba", "coordenadas": {"srid": 4326, "x": "-58.483554", "y": "-34.584619"}, "direccion": "BARZANA 1566, CABA", "nombre_calle": "BARZANA", "nombre_calle_cruce": "", "nombre_localidad": "CABA", "nombre_partido": "CABA", "tipo": "calle_altura"}]}</t>
+        </is>
+      </c>
+      <c r="K18" t="n">
+        <v>-58.483554</v>
+      </c>
+      <c r="L18" t="n">
+        <v>-34.584619</v>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>Paternal</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>Capital Norte</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">9190 </t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>5/13/2026</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>14 DE JULIO 1303</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>15</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>PENDIENTE ADMIN</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Optical Power</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>NORMALIZAR RED A BAJA ALTURA</t>
+        </is>
+      </c>
+      <c r="I19" t="n">
+        <v>1</v>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>{"direccionesNormalizadas": [{"altura": 1303, "cod_calle": 3102, "cod_calle_cruce": null, "cod_partido": "caba", "coordenadas": {"srid": 4326, "x": "-58.461808", "y": "-34.578166"}, "direccion": "14 DE JULIO 1303, CABA", "nombre_calle": "14 DE JULIO", "nombre_calle_cruce": "", "nombre_localidad": "CABA", "nombre_partido": "CABA", "tipo": "calle_altura"}]}</t>
+        </is>
+      </c>
+      <c r="K19" t="n">
+        <v>-58.461808</v>
+      </c>
+      <c r="L19" t="n">
+        <v>-34.578166</v>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>Colegiales</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>Capital Norte</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">900009976010 </t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>5/13/2026</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>JUNCAL 1887</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>3</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>PENDIENTE ADMIN</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Optical Power</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>NORMALIZAR CABLES A BAJA ALTURA</t>
+        </is>
+      </c>
+      <c r="I20" t="n">
+        <v>1</v>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>{"direccionesNormalizadas": [{"altura": 1887, "cod_calle": 10014, "cod_calle_cruce": null, "cod_partido": "caba", "coordenadas": {"srid": 4326, "x": "-58.394228", "y": "-34.593596"}, "direccion": "JUNCAL 1887, CABA", "nombre_calle": "JUNCAL", "nombre_calle_cruce": "", "nombre_localidad": "CABA", "nombre_partido": "CABA", "tipo": "calle_altura"}]}</t>
+        </is>
+      </c>
+      <c r="K20" t="n">
+        <v>-58.394228</v>
+      </c>
+      <c r="L20" t="n">
+        <v>-34.593596</v>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>Recoleta</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">9922 </t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>5/13/2026</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>ESTADO DE PALESTINA 1014</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>5</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>PENDIENTE ADMIN</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Optical Power</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>NORMALIZAR CABLES A BAJA ALTURA</t>
+        </is>
+      </c>
+      <c r="I21" t="n">
+        <v>1</v>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>{"direccionesNormalizadas": [{"altura": 1014, "cod_calle": 19016, "cod_calle_cruce": null, "cod_partido": "caba", "coordenadas": {"srid": 4326, "x": "-58.425117", "y": "-34.598984"}, "direccion": "ESTADO DE PALESTINA 1014, CABA", "nombre_calle": "ESTADO DE PALESTINA", "nombre_calle_cruce": "", "nombre_localidad": "CABA", "nombre_partido": "CABA", "tipo": "calle_altura"}]}</t>
+        </is>
+      </c>
+      <c r="K21" t="n">
+        <v>-58.425117</v>
+      </c>
+      <c r="L21" t="n">
+        <v>-34.598984</v>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>Almagro</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">9990 </t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>5/13/2026</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>COPAHUE 2065</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>4</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>PENDIENTE ADMIN</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Optical Power</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>NORMALIZAR CABLES A BAJA ALTURA</t>
+        </is>
+      </c>
+      <c r="I22" t="n">
+        <v>1</v>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>{"direccionesNormalizadas": [{"altura": 2065, "cod_calle": 3162, "cod_calle_cruce": null, "cod_partido": "caba", "coordenadas": {"srid": 4326, "x": "-58.379683", "y": "-34.641191"}, "direccion": "COPAHUE 2065, CABA", "nombre_calle": "COPAHUE", "nombre_calle_cruce": "", "nombre_localidad": "CABA", "nombre_partido": "CABA", "tipo": "calle_altura"}]}</t>
+        </is>
+      </c>
+      <c r="K22" t="n">
+        <v>-58.379683</v>
+      </c>
+      <c r="L22" t="n">
+        <v>-34.641191</v>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
           <t>San Telmo</t>
         </is>
       </c>
-      <c r="N9" t="inlineStr">
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">7789 </t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>5/14/2026</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>TAGLE 2640</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>14</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>PENDIENTE ADMIN</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Optical Power</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>NORMALIZAR CABLES A BAJA ALTURA</t>
+        </is>
+      </c>
+      <c r="I23" t="n">
+        <v>1</v>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>{"direccionesNormalizadas": [{"altura": 2640, "cod_calle": 21006, "cod_calle_cruce": null, "cod_partido": "caba", "coordenadas": {"srid": 4326, "x": "-58.399601", "y": "-34.583071"}, "direccion": "TAGLE 2640, CABA", "nombre_calle": "TAGLE", "nombre_calle_cruce": "", "nombre_localidad": "CABA", "nombre_partido": "CABA", "tipo": "calle_altura"}]}</t>
+        </is>
+      </c>
+      <c r="K23" t="n">
+        <v>-58.399601</v>
+      </c>
+      <c r="L23" t="n">
+        <v>-34.583071</v>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>Recoleta</t>
+        </is>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">7993 </t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>5/14/2026</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>PUEYRREDON AV. 394</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>3</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>PENDIENTE ADMIN</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Optical Power</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>NORMALIZAR CABLES A BAJA ALTURA</t>
+        </is>
+      </c>
+      <c r="I24" t="n">
+        <v>1</v>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>{"direccionesNormalizadas": [{"altura": 394, "cod_calle": 17132, "cod_calle_cruce": null, "cod_partido": "caba", "coordenadas": {"srid": 4326, "x": "-58.405850", "y": "-34.605697"}, "direccion": "PUEYRREDON AV. 394, CABA", "nombre_calle": "PUEYRREDON AV.", "nombre_calle_cruce": "", "nombre_localidad": "CABA", "nombre_partido": "CABA", "tipo": "calle_altura"}, {"altura": 394, "cod_calle": 17133, "cod_calle_cruce": null, "cod_partido": "caba", "coordenadas": {"srid": 4326, "x": "-58.440806", "y": "-34.615134"}, "direccion": "PUEYRREDON, HONORIO, DR. AV. 394, CABA", "nombre_calle": "PUEYRREDON, HONORIO, DR. AV.", "nombre_calle_cruce": "", "nombre_localidad": "CABA", "nombre_partido": "CABA", "tipo": "calle_altura"}]}</t>
+        </is>
+      </c>
+      <c r="K24" t="n">
+        <v>-58.40585</v>
+      </c>
+      <c r="L24" t="n">
+        <v>-34.605697</v>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>Almagro</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>Capital Sur</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">10051 </t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>5/14/2026</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>MOSCONI GENERAL AV. 2362</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>12</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>PENDIENTE ADMIN</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Optical Power</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>NORMALIZAR CABLES EN DESUSO Y A BAJA ALTURA</t>
+        </is>
+      </c>
+      <c r="I25" t="n">
+        <v>1</v>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>{"direccionesNormalizadas": [{"altura": 2362, "cod_calle": 13135, "cod_calle_cruce": null, "cod_partido": "caba", "coordenadas": {"srid": 4326, "x": "-58.495996", "y": "-34.582554"}, "direccion": "MOSCONI GENERAL AV. 2362, CABA", "nombre_calle": "MOSCONI GENERAL AV.", "nombre_calle_cruce": "", "nombre_localidad": "CABA", "nombre_partido": "CABA", "tipo": "calle_altura"}]}</t>
+        </is>
+      </c>
+      <c r="K25" t="n">
+        <v>-58.495996</v>
+      </c>
+      <c r="L25" t="n">
+        <v>-34.582554</v>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>Paternal</t>
+        </is>
+      </c>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>Capital Norte</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">10064 </t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>5/14/2026</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>CORDOBA AV. 5187</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>14</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>PENDIENTE ADMIN</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Optical Power</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>NORMALIZAR CABLES A BAJA ALTURA</t>
+        </is>
+      </c>
+      <c r="I26" t="n">
+        <v>1</v>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>{"direccionesNormalizadas": [{"altura": 5187, "cod_calle": 3165, "cod_calle_cruce": null, "cod_partido": "caba", "coordenadas": {"srid": 4326, "x": "-58.435882", "y": "-34.590339"}, "direccion": "CORDOBA AV. 5187, CABA", "nombre_calle": "CORDOBA AV.", "nombre_calle_cruce": "", "nombre_localidad": "CABA", "nombre_partido": "CABA", "tipo": "calle_altura"}]}</t>
+        </is>
+      </c>
+      <c r="K26" t="n">
+        <v>-58.435882</v>
+      </c>
+      <c r="L26" t="n">
+        <v>-34.590339</v>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>Palermo</t>
+        </is>
+      </c>
+      <c r="N26" t="inlineStr">
         <is>
           <t>Capital Sur</t>
         </is>

</xml_diff>

<commit_message>
Actualizacion automatica del mapa (2026-06-10 16:02:33)
</commit_message>
<xml_diff>
--- a/mapa_interactivo_Optical_Power.xlsx
+++ b/mapa_interactivo_Optical_Power.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N26"/>
+  <dimension ref="A1:N14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -675,21 +675,21 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>9073</t>
+          <t>9094</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>4/30/2026</t>
+          <t>5/10/2026</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>EL SALVADOR 5897</t>
+          <t>CARRIL, SALVADOR MARIA DEL AV. 3236</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -716,44 +716,44 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>{"direccionesNormalizadas": [{"altura": 5897, "cod_calle": 5050, "cod_calle_cruce": null, "cod_partido": "caba", "coordenadas": {"srid": 4326, "x": "-58.438216", "y": "-34.580964"}, "direccion": "EL SALVADOR 5897, CABA", "nombre_calle": "EL SALVADOR", "nombre_calle_cruce": "", "nombre_localidad": "CABA", "nombre_partido": "CABA", "tipo": "calle_altura"}]}</t>
+          <t>{"direccionesNormalizadas": [{"altura": 3236, "cod_calle": 4039, "cod_calle_cruce": null, "cod_partido": "caba", "coordenadas": {"srid": 4326, "x": "-58.502582", "y": "-34.593476"}, "direccion": "CARRIL, SALVADOR MARIA DEL AV. 3236, CABA", "nombre_calle": "CARRIL, SALVADOR MARIA DEL AV.", "nombre_calle_cruce": "", "nombre_localidad": "CABA", "nombre_partido": "CABA", "tipo": "calle_altura"}]}</t>
         </is>
       </c>
       <c r="K5" t="n">
-        <v>-58.438216</v>
+        <v>-58.502582</v>
       </c>
       <c r="L5" t="n">
-        <v>-34.580964</v>
+        <v>-34.593476</v>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>Palermo</t>
+          <t>Paternal</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>9094</t>
+          <t>S00415298</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>5/10/2026</t>
+          <t>5/13/2026</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>CARRIL, SALVADOR MARIA DEL AV. 3236</t>
+          <t>CARDOSO 17</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -772,7 +772,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>NORMALIZAR CABLES A BAJA ALTURA</t>
+          <t>NORMALIZAR TENDIDO A BAJA ALTURA</t>
         </is>
       </c>
       <c r="I6" t="n">
@@ -780,18 +780,18 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>{"direccionesNormalizadas": [{"altura": 3236, "cod_calle": 4039, "cod_calle_cruce": null, "cod_partido": "caba", "coordenadas": {"srid": 4326, "x": "-58.502582", "y": "-34.593476"}, "direccion": "CARRIL, SALVADOR MARIA DEL AV. 3236, CABA", "nombre_calle": "CARRIL, SALVADOR MARIA DEL AV.", "nombre_calle_cruce": "", "nombre_localidad": "CABA", "nombre_partido": "CABA", "tipo": "calle_altura"}]}</t>
+          <t>{"direccionesNormalizadas": [{"altura": 17, "cod_calle": 3070, "cod_calle_cruce": null, "cod_partido": "caba", "coordenadas": {"srid": 4326, "x": "-58.492138", "y": "-34.635993"}, "direccion": "CARDOSO 17, CABA", "nombre_calle": "CARDOSO", "nombre_calle_cruce": "", "nombre_localidad": "CABA", "nombre_partido": "CABA", "tipo": "calle_altura"}]}</t>
         </is>
       </c>
       <c r="K6" t="n">
-        <v>-58.502582</v>
+        <v>-58.492138</v>
       </c>
       <c r="L6" t="n">
-        <v>-34.593476</v>
+        <v>-34.635993</v>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>Devoto</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
@@ -803,21 +803,21 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>9128</t>
+          <t xml:space="preserve">9153 </t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>5/10/2026</t>
+          <t>5/14/2026</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>ECHEVERRIA 5596</t>
+          <t>ALVAREZ THOMAS AV. 1720</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -844,18 +844,18 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>{"direccionesNormalizadas": [{"altura": 5596, "cod_calle": 5007, "cod_calle_cruce": null, "cod_partido": "caba", "coordenadas": {"srid": 4326, "x": "-58.486598", "y": "-34.582134"}, "direccion": "ECHEVERRIA 5596, CABA", "nombre_calle": "ECHEVERRIA", "nombre_calle_cruce": "", "nombre_localidad": "CABA", "nombre_partido": "CABA", "tipo": "calle_altura"}]}</t>
+          <t>{"direccionesNormalizadas": [{"altura": 1720, "cod_calle": 1059, "cod_calle_cruce": null, "cod_partido": "caba", "coordenadas": {"srid": 4326, "x": "-58.466347", "y": "-34.579162"}, "direccion": "ALVAREZ THOMAS AV. 1720, CABA", "nombre_calle": "ALVAREZ THOMAS AV.", "nombre_calle_cruce": "", "nombre_localidad": "CABA", "nombre_partido": "CABA", "tipo": "calle_altura"}]}</t>
         </is>
       </c>
       <c r="K7" t="n">
-        <v>-58.486598</v>
+        <v>-58.466347</v>
       </c>
       <c r="L7" t="n">
-        <v>-34.582134</v>
+        <v>-34.579162</v>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>Colegiales</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -867,7 +867,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t xml:space="preserve">9141 </t>
+          <t xml:space="preserve">9158 </t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -877,11 +877,11 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>CUBAS, JOSE 4440</t>
+          <t>FRANCO 2415</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -900,7 +900,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>DESMONTAR CABLES CORTADOS Y DESMONTAR POSTE INCLINADO</t>
+          <t>MORMALIZAR TENDIDO A BAJA ALTURA</t>
         </is>
       </c>
       <c r="I8" t="n">
@@ -908,14 +908,14 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>{"direccionesNormalizadas": [{"altura": 4440, "cod_calle": 3198, "cod_calle_cruce": null, "cod_partido": "caba", "coordenadas": {"srid": 4326, "x": "-58.519391", "y": "-34.600472"}, "direccion": "CUBAS, JOSE 4440, CABA", "nombre_calle": "CUBAS, JOSE", "nombre_calle_cruce": "", "nombre_localidad": "CABA", "nombre_partido": "CABA", "tipo": "calle_altura"}]}</t>
+          <t>{"direccionesNormalizadas": [{"altura": 2415, "cod_calle": 6052, "cod_calle_cruce": null, "cod_partido": "caba", "coordenadas": {"srid": 4326, "x": "-58.501083", "y": "-34.578059"}, "direccion": "FRANCO 2415, CABA", "nombre_calle": "FRANCO", "nombre_calle_cruce": "", "nombre_localidad": "CABA", "nombre_partido": "CABA", "tipo": "calle_altura"}]}</t>
         </is>
       </c>
       <c r="K8" t="n">
-        <v>-58.519391</v>
+        <v>-58.501083</v>
       </c>
       <c r="L8" t="n">
-        <v>-34.600472</v>
+        <v>-34.578059</v>
       </c>
       <c r="M8" t="inlineStr">
         <is>
@@ -931,7 +931,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>S00347551</t>
+          <t xml:space="preserve">9159 </t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -941,11 +941,11 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>BILBAO, FRANCISCO 2124</t>
+          <t>BAZURCO 2442</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -964,7 +964,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>NORMALIZAR CABLES A BAJA ALTURA</t>
+          <t>NORMALIZAR TENDIDO A BAJA ALTURA</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -972,30 +972,30 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>{"direccionesNormalizadas": [{"altura": 2124, "cod_calle": 2081, "cod_calle_cruce": null, "cod_partido": "caba", "coordenadas": {"srid": 4326, "x": "-58.456407", "y": "-34.633376"}, "direccion": "BILBAO, FRANCISCO 2124, CABA", "nombre_calle": "BILBAO, FRANCISCO", "nombre_calle_cruce": "", "nombre_localidad": "CABA", "nombre_partido": "CABA", "tipo": "calle_altura"}]}</t>
+          <t>{"direccionesNormalizadas": [{"altura": 2442, "cod_calle": 2038, "cod_calle_cruce": null, "cod_partido": "caba", "coordenadas": {"srid": 4326, "x": "-58.502043", "y": "-34.577603"}, "direccion": "BAZURCO 2442, CABA", "nombre_calle": "BAZURCO", "nombre_calle_cruce": "", "nombre_localidad": "CABA", "nombre_partido": "CABA", "tipo": "calle_altura"}]}</t>
         </is>
       </c>
       <c r="K9" t="n">
-        <v>-58.456407</v>
+        <v>-58.502043</v>
       </c>
       <c r="L9" t="n">
-        <v>-34.633376</v>
+        <v>-34.577603</v>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>Boedo</t>
+          <t>Paternal</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>Capital Sur</t>
+          <t>Capital Norte</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>S00415298</t>
+          <t>9160</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1005,11 +1005,11 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>CARDOSO 17</t>
+          <t>CARACAS 5377</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -1028,7 +1028,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>NORMALIZAR TENDIDO A BAJA ALTURA</t>
+          <t>NORMALIZAR RED A BAJA ALTURA</t>
         </is>
       </c>
       <c r="I10" t="n">
@@ -1036,18 +1036,18 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>{"direccionesNormalizadas": [{"altura": 17, "cod_calle": 3070, "cod_calle_cruce": null, "cod_partido": "caba", "coordenadas": {"srid": 4326, "x": "-58.492138", "y": "-34.635993"}, "direccion": "CARDOSO 17, CABA", "nombre_calle": "CARDOSO", "nombre_calle_cruce": "", "nombre_localidad": "CABA", "nombre_partido": "CABA", "tipo": "calle_altura"}]}</t>
+          <t>{"direccionesNormalizadas": [{"altura": 5377, "cod_calle": 3062, "cod_calle_cruce": null, "cod_partido": "caba", "coordenadas": {"srid": 4326, "x": "-58.500199", "y": "-34.576706"}, "direccion": "CARACAS 5377, CABA", "nombre_calle": "CARACAS", "nombre_calle_cruce": "", "nombre_localidad": "CABA", "nombre_partido": "CABA", "tipo": "calle_altura"}]}</t>
         </is>
       </c>
       <c r="K10" t="n">
-        <v>-58.492138</v>
+        <v>-58.500199</v>
       </c>
       <c r="L10" t="n">
-        <v>-34.635993</v>
+        <v>-34.576706</v>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>Devoto</t>
+          <t>Paternal</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
@@ -1059,7 +1059,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>S00435575</t>
+          <t xml:space="preserve">9185 </t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1069,11 +1069,11 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>LAMAS, ANDRES 1720</t>
+          <t>CAMARGO 1157</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -1092,7 +1092,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>NORMALIZAR CABLES A BAJA ALTURA</t>
+          <t>NORMALIZAR RED A BAJA ALTURA</t>
         </is>
       </c>
       <c r="I11" t="n">
@@ -1100,14 +1100,14 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>{"direccionesNormalizadas": [{"altura": 1720, "cod_calle": 12040, "cod_calle_cruce": null, "cod_partido": "caba", "coordenadas": {"srid": 4326, "x": "-58.467729", "y": "-34.609182"}, "direccion": "LAMAS, ANDRES 1720, CABA", "nombre_calle": "LAMAS, ANDRES", "nombre_calle_cruce": "", "nombre_localidad": "CABA", "nombre_partido": "CABA", "tipo": "calle_altura"}]}</t>
+          <t>{"direccionesNormalizadas": [{"altura": 1157, "cod_calle": 3033, "cod_calle_cruce": null, "cod_partido": "caba", "coordenadas": {"srid": 4326, "x": "-58.445853", "y": "-34.595224"}, "direccion": "CAMARGO 1157, CABA", "nombre_calle": "CAMARGO", "nombre_calle_cruce": "", "nombre_localidad": "CABA", "nombre_partido": "CABA", "tipo": "calle_altura"}]}</t>
         </is>
       </c>
       <c r="K11" t="n">
-        <v>-58.467729</v>
+        <v>-58.445853</v>
       </c>
       <c r="L11" t="n">
-        <v>-34.609182</v>
+        <v>-34.595224</v>
       </c>
       <c r="M11" t="inlineStr">
         <is>
@@ -1123,7 +1123,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>S00456441</t>
+          <t xml:space="preserve">900009976010 </t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1133,11 +1133,11 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>QUESADA 4154</t>
+          <t>JUNCAL 1887</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -1156,7 +1156,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>CORTAR CABLES EN DESUSO Y VERIFICAR ESTADO COLUMNA, DOCUMENTAR CON FOTOS</t>
+          <t>NORMALIZAR CABLES A BAJA ALTURA</t>
         </is>
       </c>
       <c r="I12" t="n">
@@ -1164,30 +1164,30 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>{"direccionesNormalizadas": [{"altura": 4154, "cod_calle": 18005, "cod_calle_cruce": null, "cod_partido": "caba", "coordenadas": {"srid": 4326, "x": "-58.481018", "y": "-34.563694"}, "direccion": "QUESADA 4154, CABA", "nombre_calle": "QUESADA", "nombre_calle_cruce": "", "nombre_localidad": "CABA", "nombre_partido": "CABA", "tipo": "calle_altura"}]}</t>
+          <t>{"direccionesNormalizadas": [{"altura": 1887, "cod_calle": 10014, "cod_calle_cruce": null, "cod_partido": "caba", "coordenadas": {"srid": 4326, "x": "-58.394228", "y": "-34.593596"}, "direccion": "JUNCAL 1887, CABA", "nombre_calle": "JUNCAL", "nombre_calle_cruce": "", "nombre_localidad": "CABA", "nombre_partido": "CABA", "tipo": "calle_altura"}]}</t>
         </is>
       </c>
       <c r="K12" t="n">
-        <v>-58.481018</v>
+        <v>-58.394228</v>
       </c>
       <c r="L12" t="n">
-        <v>-34.563694</v>
+        <v>-34.593596</v>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>Saavedra</t>
+          <t>Recoleta</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>Capital Norte</t>
+          <t>Capital Sur</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t xml:space="preserve">9153 </t>
+          <t xml:space="preserve">10051 </t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1197,11 +1197,11 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>ALVAREZ THOMAS AV. 1720</t>
+          <t>MOSCONI GENERAL AV. 2362</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -1220,7 +1220,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>NORMALIZAR CABLES A BAJA ALTURA</t>
+          <t>NORMALIZAR CABLES EN DESUSO Y A BAJA ALTURA</t>
         </is>
       </c>
       <c r="I13" t="n">
@@ -1228,18 +1228,18 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>{"direccionesNormalizadas": [{"altura": 1720, "cod_calle": 1059, "cod_calle_cruce": null, "cod_partido": "caba", "coordenadas": {"srid": 4326, "x": "-58.466347", "y": "-34.579162"}, "direccion": "ALVAREZ THOMAS AV. 1720, CABA", "nombre_calle": "ALVAREZ THOMAS AV.", "nombre_calle_cruce": "", "nombre_localidad": "CABA", "nombre_partido": "CABA", "tipo": "calle_altura"}]}</t>
+          <t>{"direccionesNormalizadas": [{"altura": 2362, "cod_calle": 13135, "cod_calle_cruce": null, "cod_partido": "caba", "coordenadas": {"srid": 4326, "x": "-58.495996", "y": "-34.582554"}, "direccion": "MOSCONI GENERAL AV. 2362, CABA", "nombre_calle": "MOSCONI GENERAL AV.", "nombre_calle_cruce": "", "nombre_localidad": "CABA", "nombre_partido": "CABA", "tipo": "calle_altura"}]}</t>
         </is>
       </c>
       <c r="K13" t="n">
-        <v>-58.466347</v>
+        <v>-58.495996</v>
       </c>
       <c r="L13" t="n">
-        <v>-34.579162</v>
+        <v>-34.582554</v>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>Colegiales</t>
+          <t>Paternal</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
@@ -1251,21 +1251,21 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t xml:space="preserve">9158 </t>
+          <t xml:space="preserve">10064 </t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>5/13/2026</t>
+          <t>5/14/2026</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>FRANCO 2415</t>
+          <t>CORDOBA AV. 5187</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -1284,7 +1284,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>MORMALIZAR TENDIDO A BAJA ALTURA</t>
+          <t>NORMALIZAR CABLES A BAJA ALTURA</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -1292,789 +1292,21 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>{"direccionesNormalizadas": [{"altura": 2415, "cod_calle": 6052, "cod_calle_cruce": null, "cod_partido": "caba", "coordenadas": {"srid": 4326, "x": "-58.501083", "y": "-34.578059"}, "direccion": "FRANCO 2415, CABA", "nombre_calle": "FRANCO", "nombre_calle_cruce": "", "nombre_localidad": "CABA", "nombre_partido": "CABA", "tipo": "calle_altura"}]}</t>
+          <t>{"direccionesNormalizadas": [{"altura": 5187, "cod_calle": 3165, "cod_calle_cruce": null, "cod_partido": "caba", "coordenadas": {"srid": 4326, "x": "-58.435882", "y": "-34.590339"}, "direccion": "CORDOBA AV. 5187, CABA", "nombre_calle": "CORDOBA AV.", "nombre_calle_cruce": "", "nombre_localidad": "CABA", "nombre_partido": "CABA", "tipo": "calle_altura"}]}</t>
         </is>
       </c>
       <c r="K14" t="n">
-        <v>-58.501083</v>
+        <v>-58.435882</v>
       </c>
       <c r="L14" t="n">
-        <v>-34.578059</v>
+        <v>-34.590339</v>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>Paternal</t>
+          <t>Palermo</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
-        <is>
-          <t>Capital Norte</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">9159 </t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>5/13/2026</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>BAZURCO 2442</t>
-        </is>
-      </c>
-      <c r="D15" t="n">
-        <v>12</v>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>PENDIENTE ADMIN</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>Optical Power</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>NORMALIZAR TENDIDO A BAJA ALTURA</t>
-        </is>
-      </c>
-      <c r="I15" t="n">
-        <v>1</v>
-      </c>
-      <c r="J15" t="inlineStr">
-        <is>
-          <t>{"direccionesNormalizadas": [{"altura": 2442, "cod_calle": 2038, "cod_calle_cruce": null, "cod_partido": "caba", "coordenadas": {"srid": 4326, "x": "-58.502043", "y": "-34.577603"}, "direccion": "BAZURCO 2442, CABA", "nombre_calle": "BAZURCO", "nombre_calle_cruce": "", "nombre_localidad": "CABA", "nombre_partido": "CABA", "tipo": "calle_altura"}]}</t>
-        </is>
-      </c>
-      <c r="K15" t="n">
-        <v>-58.502043</v>
-      </c>
-      <c r="L15" t="n">
-        <v>-34.577603</v>
-      </c>
-      <c r="M15" t="inlineStr">
-        <is>
-          <t>Paternal</t>
-        </is>
-      </c>
-      <c r="N15" t="inlineStr">
-        <is>
-          <t>Capital Norte</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>9160</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>5/13/2026</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>CARACAS 5377</t>
-        </is>
-      </c>
-      <c r="D16" t="n">
-        <v>12</v>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>PENDIENTE ADMIN</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>Optical Power</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>NORMALIZAR RED A BAJA ALTURA</t>
-        </is>
-      </c>
-      <c r="I16" t="n">
-        <v>1</v>
-      </c>
-      <c r="J16" t="inlineStr">
-        <is>
-          <t>{"direccionesNormalizadas": [{"altura": 5377, "cod_calle": 3062, "cod_calle_cruce": null, "cod_partido": "caba", "coordenadas": {"srid": 4326, "x": "-58.500199", "y": "-34.576706"}, "direccion": "CARACAS 5377, CABA", "nombre_calle": "CARACAS", "nombre_calle_cruce": "", "nombre_localidad": "CABA", "nombre_partido": "CABA", "tipo": "calle_altura"}]}</t>
-        </is>
-      </c>
-      <c r="K16" t="n">
-        <v>-58.500199</v>
-      </c>
-      <c r="L16" t="n">
-        <v>-34.576706</v>
-      </c>
-      <c r="M16" t="inlineStr">
-        <is>
-          <t>Paternal</t>
-        </is>
-      </c>
-      <c r="N16" t="inlineStr">
-        <is>
-          <t>Capital Norte</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">9185 </t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>5/13/2026</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>CAMARGO 1157</t>
-        </is>
-      </c>
-      <c r="D17" t="n">
-        <v>15</v>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>PENDIENTE ADMIN</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>Optical Power</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>NORMALIZAR RED A BAJA ALTURA</t>
-        </is>
-      </c>
-      <c r="I17" t="n">
-        <v>1</v>
-      </c>
-      <c r="J17" t="inlineStr">
-        <is>
-          <t>{"direccionesNormalizadas": [{"altura": 1157, "cod_calle": 3033, "cod_calle_cruce": null, "cod_partido": "caba", "coordenadas": {"srid": 4326, "x": "-58.445853", "y": "-34.595224"}, "direccion": "CAMARGO 1157, CABA", "nombre_calle": "CAMARGO", "nombre_calle_cruce": "", "nombre_localidad": "CABA", "nombre_partido": "CABA", "tipo": "calle_altura"}]}</t>
-        </is>
-      </c>
-      <c r="K17" t="n">
-        <v>-58.445853</v>
-      </c>
-      <c r="L17" t="n">
-        <v>-34.595224</v>
-      </c>
-      <c r="M17" t="inlineStr">
-        <is>
-          <t>Paternal</t>
-        </is>
-      </c>
-      <c r="N17" t="inlineStr">
-        <is>
-          <t>Capital Norte</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">9188 </t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>5/13/2026</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>BARZANA 1566</t>
-        </is>
-      </c>
-      <c r="D18" t="n">
-        <v>12</v>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>PENDIENTE ADMIN</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>Optical Power</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>NORMALIZAR RED A BAJA ALTURA</t>
-        </is>
-      </c>
-      <c r="I18" t="n">
-        <v>1</v>
-      </c>
-      <c r="J18" t="inlineStr">
-        <is>
-          <t>{"direccionesNormalizadas": [{"altura": 1566, "cod_calle": 2023, "cod_calle_cruce": null, "cod_partido": "caba", "coordenadas": {"srid": 4326, "x": "-58.483554", "y": "-34.584619"}, "direccion": "BARZANA 1566, CABA", "nombre_calle": "BARZANA", "nombre_calle_cruce": "", "nombre_localidad": "CABA", "nombre_partido": "CABA", "tipo": "calle_altura"}]}</t>
-        </is>
-      </c>
-      <c r="K18" t="n">
-        <v>-58.483554</v>
-      </c>
-      <c r="L18" t="n">
-        <v>-34.584619</v>
-      </c>
-      <c r="M18" t="inlineStr">
-        <is>
-          <t>Paternal</t>
-        </is>
-      </c>
-      <c r="N18" t="inlineStr">
-        <is>
-          <t>Capital Norte</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t xml:space="preserve">9190 </t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>5/13/2026</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>14 DE JULIO 1303</t>
-        </is>
-      </c>
-      <c r="D19" t="n">
-        <v>15</v>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>PENDIENTE ADMIN</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>Optical Power</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>NORMALIZAR RED A BAJA ALTURA</t>
-        </is>
-      </c>
-      <c r="I19" t="n">
-        <v>1</v>
-      </c>
-      <c r="J19" t="inlineStr">
-        <is>
-          <t>{"direccionesNormalizadas": [{"altura": 1303, "cod_calle": 3102, "cod_calle_cruce": null, "cod_partido": "caba", "coordenadas": {"srid": 4326, "x": "-58.461808", "y": "-34.578166"}, "direccion": "14 DE JULIO 1303, CABA", "nombre_calle": "14 DE JULIO", "nombre_calle_cruce": "", "nombre_localidad": "CABA", "nombre_partido": "CABA", "tipo": "calle_altura"}]}</t>
-        </is>
-      </c>
-      <c r="K19" t="n">
-        <v>-58.461808</v>
-      </c>
-      <c r="L19" t="n">
-        <v>-34.578166</v>
-      </c>
-      <c r="M19" t="inlineStr">
-        <is>
-          <t>Colegiales</t>
-        </is>
-      </c>
-      <c r="N19" t="inlineStr">
-        <is>
-          <t>Capital Norte</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">900009976010 </t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>5/13/2026</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>JUNCAL 1887</t>
-        </is>
-      </c>
-      <c r="D20" t="n">
-        <v>3</v>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>PENDIENTE ADMIN</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>Optical Power</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>NORMALIZAR CABLES A BAJA ALTURA</t>
-        </is>
-      </c>
-      <c r="I20" t="n">
-        <v>1</v>
-      </c>
-      <c r="J20" t="inlineStr">
-        <is>
-          <t>{"direccionesNormalizadas": [{"altura": 1887, "cod_calle": 10014, "cod_calle_cruce": null, "cod_partido": "caba", "coordenadas": {"srid": 4326, "x": "-58.394228", "y": "-34.593596"}, "direccion": "JUNCAL 1887, CABA", "nombre_calle": "JUNCAL", "nombre_calle_cruce": "", "nombre_localidad": "CABA", "nombre_partido": "CABA", "tipo": "calle_altura"}]}</t>
-        </is>
-      </c>
-      <c r="K20" t="n">
-        <v>-58.394228</v>
-      </c>
-      <c r="L20" t="n">
-        <v>-34.593596</v>
-      </c>
-      <c r="M20" t="inlineStr">
-        <is>
-          <t>Recoleta</t>
-        </is>
-      </c>
-      <c r="N20" t="inlineStr">
-        <is>
-          <t>Capital Sur</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t xml:space="preserve">9922 </t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>5/13/2026</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>ESTADO DE PALESTINA 1014</t>
-        </is>
-      </c>
-      <c r="D21" t="n">
-        <v>5</v>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>PENDIENTE ADMIN</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>Optical Power</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>NORMALIZAR CABLES A BAJA ALTURA</t>
-        </is>
-      </c>
-      <c r="I21" t="n">
-        <v>1</v>
-      </c>
-      <c r="J21" t="inlineStr">
-        <is>
-          <t>{"direccionesNormalizadas": [{"altura": 1014, "cod_calle": 19016, "cod_calle_cruce": null, "cod_partido": "caba", "coordenadas": {"srid": 4326, "x": "-58.425117", "y": "-34.598984"}, "direccion": "ESTADO DE PALESTINA 1014, CABA", "nombre_calle": "ESTADO DE PALESTINA", "nombre_calle_cruce": "", "nombre_localidad": "CABA", "nombre_partido": "CABA", "tipo": "calle_altura"}]}</t>
-        </is>
-      </c>
-      <c r="K21" t="n">
-        <v>-58.425117</v>
-      </c>
-      <c r="L21" t="n">
-        <v>-34.598984</v>
-      </c>
-      <c r="M21" t="inlineStr">
-        <is>
-          <t>Almagro</t>
-        </is>
-      </c>
-      <c r="N21" t="inlineStr">
-        <is>
-          <t>Capital Sur</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t xml:space="preserve">9990 </t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>5/13/2026</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>COPAHUE 2065</t>
-        </is>
-      </c>
-      <c r="D22" t="n">
-        <v>4</v>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>PENDIENTE ADMIN</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>Optical Power</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t>NORMALIZAR CABLES A BAJA ALTURA</t>
-        </is>
-      </c>
-      <c r="I22" t="n">
-        <v>1</v>
-      </c>
-      <c r="J22" t="inlineStr">
-        <is>
-          <t>{"direccionesNormalizadas": [{"altura": 2065, "cod_calle": 3162, "cod_calle_cruce": null, "cod_partido": "caba", "coordenadas": {"srid": 4326, "x": "-58.379683", "y": "-34.641191"}, "direccion": "COPAHUE 2065, CABA", "nombre_calle": "COPAHUE", "nombre_calle_cruce": "", "nombre_localidad": "CABA", "nombre_partido": "CABA", "tipo": "calle_altura"}]}</t>
-        </is>
-      </c>
-      <c r="K22" t="n">
-        <v>-58.379683</v>
-      </c>
-      <c r="L22" t="n">
-        <v>-34.641191</v>
-      </c>
-      <c r="M22" t="inlineStr">
-        <is>
-          <t>San Telmo</t>
-        </is>
-      </c>
-      <c r="N22" t="inlineStr">
-        <is>
-          <t>Capital Sur</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t xml:space="preserve">7789 </t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>5/14/2026</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>TAGLE 2640</t>
-        </is>
-      </c>
-      <c r="D23" t="n">
-        <v>14</v>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>PENDIENTE ADMIN</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>Optical Power</t>
-        </is>
-      </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>NORMALIZAR CABLES A BAJA ALTURA</t>
-        </is>
-      </c>
-      <c r="I23" t="n">
-        <v>1</v>
-      </c>
-      <c r="J23" t="inlineStr">
-        <is>
-          <t>{"direccionesNormalizadas": [{"altura": 2640, "cod_calle": 21006, "cod_calle_cruce": null, "cod_partido": "caba", "coordenadas": {"srid": 4326, "x": "-58.399601", "y": "-34.583071"}, "direccion": "TAGLE 2640, CABA", "nombre_calle": "TAGLE", "nombre_calle_cruce": "", "nombre_localidad": "CABA", "nombre_partido": "CABA", "tipo": "calle_altura"}]}</t>
-        </is>
-      </c>
-      <c r="K23" t="n">
-        <v>-58.399601</v>
-      </c>
-      <c r="L23" t="n">
-        <v>-34.583071</v>
-      </c>
-      <c r="M23" t="inlineStr">
-        <is>
-          <t>Recoleta</t>
-        </is>
-      </c>
-      <c r="N23" t="inlineStr">
-        <is>
-          <t>Capital Sur</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t xml:space="preserve">7993 </t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>5/14/2026</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>PUEYRREDON AV. 394</t>
-        </is>
-      </c>
-      <c r="D24" t="n">
-        <v>3</v>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>PENDIENTE ADMIN</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>Optical Power</t>
-        </is>
-      </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>NORMALIZAR CABLES A BAJA ALTURA</t>
-        </is>
-      </c>
-      <c r="I24" t="n">
-        <v>1</v>
-      </c>
-      <c r="J24" t="inlineStr">
-        <is>
-          <t>{"direccionesNormalizadas": [{"altura": 394, "cod_calle": 17132, "cod_calle_cruce": null, "cod_partido": "caba", "coordenadas": {"srid": 4326, "x": "-58.405850", "y": "-34.605697"}, "direccion": "PUEYRREDON AV. 394, CABA", "nombre_calle": "PUEYRREDON AV.", "nombre_calle_cruce": "", "nombre_localidad": "CABA", "nombre_partido": "CABA", "tipo": "calle_altura"}, {"altura": 394, "cod_calle": 17133, "cod_calle_cruce": null, "cod_partido": "caba", "coordenadas": {"srid": 4326, "x": "-58.440806", "y": "-34.615134"}, "direccion": "PUEYRREDON, HONORIO, DR. AV. 394, CABA", "nombre_calle": "PUEYRREDON, HONORIO, DR. AV.", "nombre_calle_cruce": "", "nombre_localidad": "CABA", "nombre_partido": "CABA", "tipo": "calle_altura"}]}</t>
-        </is>
-      </c>
-      <c r="K24" t="n">
-        <v>-58.40585</v>
-      </c>
-      <c r="L24" t="n">
-        <v>-34.605697</v>
-      </c>
-      <c r="M24" t="inlineStr">
-        <is>
-          <t>Almagro</t>
-        </is>
-      </c>
-      <c r="N24" t="inlineStr">
-        <is>
-          <t>Capital Sur</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">10051 </t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>5/14/2026</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>MOSCONI GENERAL AV. 2362</t>
-        </is>
-      </c>
-      <c r="D25" t="n">
-        <v>12</v>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>PENDIENTE ADMIN</t>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>Optical Power</t>
-        </is>
-      </c>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="H25" t="inlineStr">
-        <is>
-          <t>NORMALIZAR CABLES EN DESUSO Y A BAJA ALTURA</t>
-        </is>
-      </c>
-      <c r="I25" t="n">
-        <v>1</v>
-      </c>
-      <c r="J25" t="inlineStr">
-        <is>
-          <t>{"direccionesNormalizadas": [{"altura": 2362, "cod_calle": 13135, "cod_calle_cruce": null, "cod_partido": "caba", "coordenadas": {"srid": 4326, "x": "-58.495996", "y": "-34.582554"}, "direccion": "MOSCONI GENERAL AV. 2362, CABA", "nombre_calle": "MOSCONI GENERAL AV.", "nombre_calle_cruce": "", "nombre_localidad": "CABA", "nombre_partido": "CABA", "tipo": "calle_altura"}]}</t>
-        </is>
-      </c>
-      <c r="K25" t="n">
-        <v>-58.495996</v>
-      </c>
-      <c r="L25" t="n">
-        <v>-34.582554</v>
-      </c>
-      <c r="M25" t="inlineStr">
-        <is>
-          <t>Paternal</t>
-        </is>
-      </c>
-      <c r="N25" t="inlineStr">
-        <is>
-          <t>Capital Norte</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">10064 </t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>5/14/2026</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>CORDOBA AV. 5187</t>
-        </is>
-      </c>
-      <c r="D26" t="n">
-        <v>14</v>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>PENDIENTE ADMIN</t>
-        </is>
-      </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>Optical Power</t>
-        </is>
-      </c>
-      <c r="G26" t="inlineStr">
-        <is>
-          <t>Pendiente</t>
-        </is>
-      </c>
-      <c r="H26" t="inlineStr">
-        <is>
-          <t>NORMALIZAR CABLES A BAJA ALTURA</t>
-        </is>
-      </c>
-      <c r="I26" t="n">
-        <v>1</v>
-      </c>
-      <c r="J26" t="inlineStr">
-        <is>
-          <t>{"direccionesNormalizadas": [{"altura": 5187, "cod_calle": 3165, "cod_calle_cruce": null, "cod_partido": "caba", "coordenadas": {"srid": 4326, "x": "-58.435882", "y": "-34.590339"}, "direccion": "CORDOBA AV. 5187, CABA", "nombre_calle": "CORDOBA AV.", "nombre_calle_cruce": "", "nombre_localidad": "CABA", "nombre_partido": "CABA", "tipo": "calle_altura"}]}</t>
-        </is>
-      </c>
-      <c r="K26" t="n">
-        <v>-58.435882</v>
-      </c>
-      <c r="L26" t="n">
-        <v>-34.590339</v>
-      </c>
-      <c r="M26" t="inlineStr">
-        <is>
-          <t>Palermo</t>
-        </is>
-      </c>
-      <c r="N26" t="inlineStr">
         <is>
           <t>Capital Sur</t>
         </is>

</xml_diff>